<commit_message>
실행 취소 / 다시 실행 (Ctrl+Z / Ctrl+Y)
- 프로젝트 상태 기록(최대 100단계, 0.4초 묶음), 편집 메뉴와 단축키
- 일지 갱신

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="158">
   <si>
     <r>
       <rPr>
@@ -5875,6 +5875,115 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">615470e</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">순위</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실행 취소 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다시 실행</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">편집 메뉴 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ Ctrl+Z / Ctrl+Y(Ctrl+Shift+Z). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">편집이 멈추고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 뒤 한 단계로 기록</t>
+    </r>
     <r>
       <rPr>
         <sz val="10"/>
@@ -5892,6 +6001,160 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">슬라이더를 끌어도 한 번</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">최대 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">새로 만들기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">열기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">복구 때 기록 초기화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 테스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 삭제 취소 → 자르기 취소 → 다시 실행 → 제목 추가 취소</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">이번 커밋</t>
     </r>
     <r>
@@ -6111,6 +6374,9 @@
       </rPr>
       <t xml:space="preserve">결과 검사 테스트 추가</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">실행 취소 기록 테스트 추가</t>
   </si>
 </sst>
 </file>
@@ -6460,8 +6726,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F26"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -6488,8 +6754,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E13"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -6712,7 +6978,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E15,"완료")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6730,7 +6996,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E15,"대기")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6739,7 +7005,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.714285714285714</v>
+        <v>0.785714285714286</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6751,8 +7017,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C25)</f>
-        <v>24</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C26)</f>
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6760,7 +7026,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B25,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B26,"사용자 제보")</f>
         <v>3</v>
       </c>
     </row>
@@ -6769,8 +7035,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B12,11)</f>
-        <v>72</v>
+        <f aca="false">INDEX(테스트!B2:B13,12)</f>
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6778,8 +7044,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C12,11)</f>
-        <v>72</v>
+        <f aca="false">INDEX(테스트!C2:C13,12)</f>
+        <v>74</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7085,9 +7351,11 @@
         <v>50</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="n">
@@ -7103,7 +7371,7 @@
         <v>53</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" s="8"/>
     </row>
@@ -7179,7 +7447,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7680,6 +7948,26 @@
       </c>
       <c r="F25" s="8" t="s">
         <v>139</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -7701,7 +7989,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7715,16 +8003,16 @@
         <v>58</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>110</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7742,7 +8030,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7760,7 +8048,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7778,7 +8066,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7796,7 +8084,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7814,7 +8102,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7832,7 +8120,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7850,7 +8138,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7868,7 +8156,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7886,7 +8174,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7904,7 +8192,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7922,7 +8210,25 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>153</v>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <f aca="false">IFERROR(C13/B13,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Beat sync: cut every N seconds and 'clip count × cut length' video length
Each clip is used exactly once for one cut, so 8 clips at 2.5 s make a
20 s video and the music ends there too. Seconds mode works without music.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="215">
   <si>
     <r>
       <rPr>
@@ -9888,6 +9888,457 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 개수 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 영상 길이</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자르는 기준</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 비트마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일정한 초마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과 영상 길이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 개수 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">컷 길이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립마다 한 컷씩</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일 순서 또는 무작위</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">노래</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영상 모두 거기서 끝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정보 줄에 완성 길이와 경고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악이 짧음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">컷보다 짧은 클립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">표시</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 2.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= 0:20.0, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미리보기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타임라인 조각 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -10219,6 +10670,55 @@
   </si>
   <si>
     <t xml:space="preserve">오류 기록 테스트 추가</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 개수 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -10426,7 +10926,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -10470,14 +10970,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEEEEEE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -10568,8 +11060,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F37"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -10596,8 +11088,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E18"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -10820,7 +11312,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"완료")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10829,7 +11321,7 @@
       </c>
       <c r="B5" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"진행 중")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10847,7 +11339,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10859,8 +11351,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C36)</f>
-        <v>35</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C37)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10868,7 +11360,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B36,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B37,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -10877,8 +11369,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B17,16)</f>
-        <v>81</v>
+        <f aca="false">INDEX(테스트!B2:B18,17)</f>
+        <v>83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10886,8 +11378,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C17,16)</f>
-        <v>81</v>
+        <f aca="false">INDEX(테스트!C2:C18,17)</f>
+        <v>83</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11369,9 +11861,11 @@
         <v>69</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F21" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="n">
@@ -11465,19 +11959,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E26">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"진행 중"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"대기"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"수정"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"확인 대기"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11499,7 +11993,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -12208,9 +12702,27 @@
         <v>191</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F36" s="8"/>
+    </row>
+    <row r="37" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="F37" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12231,7 +12743,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -12245,16 +12757,16 @@
         <v>80</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>132</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12272,7 +12784,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12290,7 +12802,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12308,7 +12820,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12326,7 +12838,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12344,7 +12856,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12362,7 +12874,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12380,7 +12892,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12398,7 +12910,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12416,7 +12928,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12434,7 +12946,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12452,7 +12964,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12470,7 +12982,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12488,7 +13000,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12506,7 +13018,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12524,7 +13036,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12542,7 +13054,25 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>210</v>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <f aca="false">IFERROR(C18/B18,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Devlog: per-clip length done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="216">
   <si>
     <r>
       <rPr>
@@ -10337,6 +10337,9 @@
       </rPr>
       <t xml:space="preserve">개</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">5b7fb40</t>
   </si>
   <si>
     <t xml:space="preserve">테스트 수</t>
@@ -12722,7 +12725,9 @@
       <c r="E37" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="F37" s="8"/>
+      <c r="F37" s="8" t="s">
+        <v>195</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12757,16 +12762,16 @@
         <v>80</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>132</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12784,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12802,7 +12807,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12820,7 +12825,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12838,7 +12843,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12856,7 +12861,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12874,7 +12879,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12892,7 +12897,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12910,7 +12915,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12928,7 +12933,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12946,7 +12951,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12964,7 +12969,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12982,7 +12987,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13000,7 +13005,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13018,7 +13023,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13036,7 +13041,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13054,7 +13059,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13072,7 +13077,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keyboard shortcuts: space play, Delete remove, F5 preview, Ctrl+E export
- Playback menu with Space, Ctrl+Left/Right (5 s), F5/Ctrl+R, Ctrl+E
- Delete/Backspace removes the selected clip, PiP, subtitle or title row
- Music gauge keeps its own Space/arrow keys; text fields keep typing
- Ignore render shortcuts while another job runs
- Fix: deleting subtitle rows now records undo/autosave

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="222">
   <si>
     <r>
       <rPr>
@@ -10340,6 +10340,379 @@
   </si>
   <si>
     <t xml:space="preserve">5b7fb40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">단축키</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재생 메뉴 추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Space </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재생</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일시정지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">글자 칸</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 게이지에서는 원래 동작</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), Ctrl+←/→ 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 이동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, F5·Ctrl+R </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미리보기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, Ctrl+E </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목 목록에서 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Delete</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 지우기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작업 중에는 단축키로 렌더링이 겹쳐 시작되지 않게 막음</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 테스트로 키 동작 확인</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">버그 수정</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 줄 삭제가 실행 취소</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자동 저장에 안 잡힘</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 탭에서 줄을 지워도 변경 알림이 없어 실행 취소 기록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자동 저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타임라인 갱신이 빠졌음 → 변경 알림 추가</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">테스트 수</t>
@@ -10929,7 +11302,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -10973,6 +11346,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEEEEEE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -11063,8 +11444,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F39"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -11315,7 +11696,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"완료")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11324,7 +11705,7 @@
       </c>
       <c r="B5" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"진행 중")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11333,7 +11714,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"대기")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11342,7 +11723,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11354,8 +11735,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C37)</f>
-        <v>36</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C39)</f>
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11363,7 +11744,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B37,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B39,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -11884,7 +12265,7 @@
         <v>71</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" s="8"/>
     </row>
@@ -11902,9 +12283,11 @@
         <v>73</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F23" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="n">
@@ -11962,19 +12345,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E26">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"완료"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"진행 중"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"대기"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"수정"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"확인 대기"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11996,7 +12379,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -12728,6 +13111,42 @@
       <c r="F37" s="8" t="s">
         <v>195</v>
       </c>
+    </row>
+    <row r="38" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="F39" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12762,16 +13181,16 @@
         <v>80</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>132</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12789,7 +13208,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12807,7 +13226,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12825,7 +13244,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12843,7 +13262,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12861,7 +13280,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12879,7 +13298,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12897,7 +13316,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12915,7 +13334,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12933,7 +13352,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12951,7 +13370,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12969,7 +13388,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12987,7 +13406,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13005,7 +13424,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13023,7 +13442,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13041,7 +13460,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13059,7 +13478,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13077,7 +13496,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ken Burns motion for photos; 10-minute stress test results
- Clip.motion: auto (alternates zoom in / pan right / zoom out / pan left),
  zoom_in, zoom_out, pan_left, pan_right, none
- Photo is upscaled once (3x) and zoompan crops each frame for smooth motion;
  shorter cuts move less (4-15%)
- Stress test: 1281 beat cuts over 600 s render exactly, cuts stay on beat

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="229">
   <si>
     <r>
       <rPr>
@@ -10715,6 +10715,855 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">대규모 프로젝트 스트레스 테스트</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">720p </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ 10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분 음악</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(128 BPM), 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트마다 컷 → 조각 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1281</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">120</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">줄</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">렌더링 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">520</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">코어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다른 작업과 동시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메모리 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">178MB(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">앱</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)·462MB(ffmpeg). 9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 이후에도 컷이 비트와 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프레임 이내</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중앙값 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.7ms), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">끝부분 소리 어긋남 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">±20ms </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이내</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 600.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 정확</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">사진 켄 번즈 효과</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립마다 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 움직임</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확대→오른쪽→축소→왼쪽 번갈아</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확대</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">축소</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">좌우 이동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">없음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진을 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배로 한 번 키운 뒤 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">zoompan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">으로 잘라내 떨림 없이 움직임</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">짧은 컷일수록 덜 움직임</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(4%~15%). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 렌더링 시간은 약 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1080×1920 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9.5→21</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -11075,6 +11924,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">초 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 움직임 테스트 </t>
     </r>
     <r>
       <rPr>
@@ -11302,7 +12181,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -11346,14 +12225,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEEEEEE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -11444,8 +12315,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F41"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -11472,8 +12343,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E19"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -11696,7 +12567,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"완료")</f>
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11705,7 +12576,7 @@
       </c>
       <c r="B5" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"진행 중")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11714,7 +12585,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"대기")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11723,7 +12594,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.76</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11735,8 +12606,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C39)</f>
-        <v>38</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C41)</f>
+        <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11744,7 +12615,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B39,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B41,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -11753,8 +12624,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B18,17)</f>
-        <v>83</v>
+        <f aca="false">INDEX(테스트!B2:B19,18)</f>
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11762,8 +12633,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C18,17)</f>
-        <v>83</v>
+        <f aca="false">INDEX(테스트!C2:C19,18)</f>
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12265,9 +13136,11 @@
         <v>71</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F22" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="n">
@@ -12303,9 +13176,11 @@
         <v>75</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F24" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="n">
@@ -12345,19 +13220,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E26">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"진행 중"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"대기"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"수정"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"확인 대기"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12379,7 +13254,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -13147,6 +14022,42 @@
         <v>93</v>
       </c>
       <c r="F39" s="8"/>
+    </row>
+    <row r="40" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F41" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -13167,7 +14078,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -13181,16 +14092,16 @@
         <v>80</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>132</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13208,7 +14119,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13226,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13244,7 +14155,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13262,7 +14173,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13280,7 +14191,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13298,7 +14209,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13316,7 +14227,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13334,7 +14245,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13352,7 +14263,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13370,7 +14281,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13388,7 +14299,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13406,7 +14317,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13424,7 +14335,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13442,7 +14353,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13460,7 +14371,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13478,7 +14389,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13496,7 +14407,25 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>221</v>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <f aca="false">IFERROR(C19/B19,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Music ducking: lower the music while clips or PiP have speech
- MusicSettings.duck: off | light | normal | strong (about 9/13/18 dB for normal speech)
- Clip + PiP audio is mixed first and drives sidechaincompress on the music
- Music tab control; e2e test measures the reduction on a real render

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="233">
   <si>
     <r>
       <rPr>
@@ -11564,6 +11564,401 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">말할 때 음악 자동 줄이기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">덕킹</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 탭 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">말할 때 음악 줄이기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">줄이지 않음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">약하게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보통</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면 소리를 섞어 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">sidechaincompress</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 음악을 누름</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(120Hz </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아래 웅웅거림은 무시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실제 크기로 맞춰 보니 처음 값은 너무 약했음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">최대 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.6dB) → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보통 말소리 기준 약 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9/13/18dB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 다시 맞춤</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. -40dB </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아래 잡음에는 반응 안 함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악이 영상보다 짧을 때</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면 소리 섞을 때도 확인</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실측 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8.8/13.0/17.4dB</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -11973,6 +12368,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">개 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">덕킹 그래프</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실제 렌더링 측정 테스트 추가</t>
     </r>
   </si>
 </sst>
@@ -12315,8 +12740,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F42"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -12343,8 +12768,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E20"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -12567,7 +12992,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"완료")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12585,7 +13010,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E26,"대기")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12594,7 +13019,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12606,8 +13031,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C41)</f>
-        <v>40</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C42)</f>
+        <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12615,7 +13040,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B41,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B42,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -12624,8 +13049,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B19,18)</f>
-        <v>85</v>
+        <f aca="false">INDEX(테스트!B2:B20,19)</f>
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12633,8 +13058,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C19,18)</f>
-        <v>85</v>
+        <f aca="false">INDEX(테스트!C2:C20,19)</f>
+        <v>87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13196,9 +13621,11 @@
         <v>77</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F25" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="n">
@@ -13254,7 +13681,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -14058,6 +14485,24 @@
         <v>207</v>
       </c>
       <c r="F41" s="8"/>
+    </row>
+    <row r="42" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="F42" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -14078,7 +14523,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -14092,16 +14537,16 @@
         <v>80</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>132</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14119,7 +14564,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14137,7 +14582,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14155,7 +14600,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14173,7 +14618,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14191,7 +14636,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14209,7 +14654,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14227,7 +14672,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14245,7 +14690,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14263,7 +14708,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14281,7 +14726,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14299,7 +14744,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14317,7 +14762,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14335,7 +14780,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14353,7 +14798,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14371,7 +14816,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14389,7 +14834,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14407,7 +14852,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14425,7 +14870,25 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>228</v>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <f aca="false">IFERROR(C20/B20,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Color filters and GPU encoding with CPU fallback
- Export color: warm, cool (colortemperature), vivid, vintage, black and white;
  applied before subtitles/titles so text keeps its color
- Export uses NVENC/QSV/AMF when a quick probe encode works; on failure it
  logs, retries with libx264 and stops using that encoder for the session
- Speed box defaults to 1x before a clip is selected

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="253">
   <si>
     <r>
       <rPr>
@@ -2124,6 +2124,240 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래픽카드 인코딩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(NVIDIA·Intel·AMD) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자동 사용</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기가 가장 오래 걸리는 단계 — 그래픽카드가 있는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 체감 속도가 크게 좋아짐</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브 한 번에 둘 다 내보내기</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">같은 영상을 비율만 바꿔 두 번 올리는 경우가 많음 — 설정 바꾸고 다시 내보내는 반복을 줄임</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대표 이미지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">썸네일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">저장</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">유튜브 업로드에 필요 — 미리보기에서 원하는 장면을 바로 이미지로</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 등장 효과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">톡 튀어나오기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">페이드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 자막에서 흔한 연출</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완성도 향상</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">날짜</t>
   </si>
   <si>
@@ -11959,6 +12193,918 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">색감 필터</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">색감</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">따뜻하게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차갑게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선명하게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빈티지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">흑백</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목보다 먼저 적용해서 글자 색은 그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">처음 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">colorbalance </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값은 눈에 거의 안 띄어서 따뜻하게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차갑게는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">colortemperature(4500K/9000K)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 바꿈</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가지 비교 이미지 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모든 색감 실제 렌더링 테스트</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 로드맵</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20~25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">26 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래픽카드 인코딩</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">속도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), 27 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브 동시 내보내기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반복 줄이기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), 28 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">썸네일 저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 29 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 등장 효과</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">그래픽카드 인코딩</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래픽카드로 빠르게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기본 켬</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">): NVIDIA→Intel→AMD </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">순으로 작은 영상을 실제 인코딩해 보고 되는 것 사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">한 번만 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">최종 영상만 그래픽카드로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">조각은 캐시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정확한 프레임 수 때문에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실패하면 오류 기록 남기고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 자동 재시도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이번 실행 동안 그 인코더는 다시 안 씀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 메시지에 사용한 그래픽카드 표시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 개발 환경엔 그래픽카드가 없어 실패→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재시도 흐름으로 확인</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실제 그래픽카드 확인은 사용자 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">필요</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 선택 전 속도 칸이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배로 보임</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립을 고르기 전 비활성 속도 칸이 첫 항목</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(0.25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">으로 보여 헷갈림 → 기본 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배로</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -12398,6 +13544,66 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">실제 렌더링 측정 테스트 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">색감 필터 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래픽카드 실패→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재시도 테스트 등 추가</t>
     </r>
   </si>
 </sst>
@@ -12740,8 +13946,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F46"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -12754,8 +13960,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F30"/>
   <tableColumns count="6">
     <tableColumn id="1" name="순위"/>
     <tableColumn id="2" name="항목"/>
@@ -12768,8 +13974,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E22"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -12982,8 +14188,8 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <f aca="false">COUNTA(로드맵!B2:B26)</f>
-        <v>25</v>
+        <f aca="false">COUNTA(로드맵!B2:B30)</f>
+        <v>29</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12991,8 +14197,8 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E26,"완료")</f>
-        <v>22</v>
+        <f aca="false">COUNTIF(로드맵!E2:E30,"완료")</f>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13000,7 +14206,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E26,"진행 중")</f>
+        <f aca="false">COUNTIF(로드맵!E2:E30,"진행 중")</f>
         <v>0</v>
       </c>
     </row>
@@ -13009,8 +14215,8 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E26,"대기")</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(로드맵!E2:E30,"대기")</f>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13019,7 +14225,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.88</v>
+        <v>0.827586206896552</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13031,8 +14237,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C42)</f>
-        <v>41</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C46)</f>
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13040,7 +14246,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B42,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B46,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -13049,8 +14255,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B20,19)</f>
-        <v>87</v>
+        <f aca="false">INDEX(테스트!B2:B22,21)</f>
+        <v>91</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13058,8 +14264,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C20,19)</f>
-        <v>87</v>
+        <f aca="false">INDEX(테스트!C2:C22,21)</f>
+        <v>91</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13120,7 +14326,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -13641,12 +14847,88 @@
         <v>79</v>
       </c>
       <c r="E26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F26" s="8"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E26">
+  <conditionalFormatting sqref="E2:E30">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
@@ -13681,7 +14963,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -13694,182 +14976,182 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13877,16 +15159,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -13895,19 +15177,19 @@
         <v>28</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13915,19 +15197,19 @@
         <v>28</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13935,19 +15217,19 @@
         <v>28</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13955,19 +15237,19 @@
         <v>28</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13975,16 +15257,16 @@
         <v>28</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -13993,19 +15275,19 @@
         <v>28</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14013,19 +15295,19 @@
         <v>28</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14033,19 +15315,19 @@
         <v>28</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14053,19 +15335,19 @@
         <v>28</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14073,19 +15355,19 @@
         <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14093,19 +15375,19 @@
         <v>28</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14113,19 +15395,19 @@
         <v>28</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14133,19 +15415,19 @@
         <v>28</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14153,13 +15435,13 @@
         <v>28</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -14169,19 +15451,19 @@
         <v>28</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14189,19 +15471,19 @@
         <v>28</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14209,19 +15491,19 @@
         <v>28</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14229,19 +15511,19 @@
         <v>28</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14249,19 +15531,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14269,13 +15551,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -14285,19 +15567,19 @@
         <v>28</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14305,19 +15587,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14325,19 +15607,19 @@
         <v>28</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14345,13 +15627,13 @@
         <v>28</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
@@ -14361,19 +15643,19 @@
         <v>28</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14381,13 +15663,13 @@
         <v>28</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>2</v>
@@ -14399,19 +15681,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14419,16 +15701,16 @@
         <v>28</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -14437,16 +15719,16 @@
         <v>28</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -14455,16 +15737,16 @@
         <v>28</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -14473,16 +15755,16 @@
         <v>28</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -14491,18 +15773,90 @@
         <v>28</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="F42" s="8"/>
+    </row>
+    <row r="43" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" customFormat="false" ht="72.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="F46" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -14523,7 +15877,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -14534,24 +15888,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>50</v>
@@ -14564,7 +15918,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>214</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14582,7 +15936,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14600,7 +15954,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>216</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14618,7 +15972,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14636,7 +15990,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14654,7 +16008,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14672,7 +16026,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14690,7 +16044,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14708,7 +16062,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14726,7 +16080,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14744,7 +16098,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14762,7 +16116,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14780,7 +16134,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>226</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14798,7 +16152,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14816,7 +16170,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14834,7 +16188,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>229</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14852,7 +16206,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14870,7 +16224,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14888,7 +16242,43 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>232</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <f aca="false">IFERROR(C21/B21,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <f aca="false">IFERROR(C22/B22,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Export several aspect ratios in one go
- Multi-export dialog (button and Ctrl+Shift+E): YouTube, Reels, square, 4:5
  at a chosen resolution, saved as name_유튜브.mp4, name_릴스.mp4, ...
- Preview/export/multi-export share one render runner with per-file progress

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="257">
   <si>
     <r>
       <rPr>
@@ -13105,6 +13105,335 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">여러 비율로 한 번에 내보내기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">📐 버튼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·Ctrl+Shift+E: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정사각형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">인스타 피드 중 고르고 해상도 선택 → 이름</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이름</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 … </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차례로 만듦</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행 표시에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[2/3] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일 이름 표시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">취소하면 남은 것도 멈춤</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미리보기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기 실행 코드를 하나로 정리</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 테스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 비율 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">720p 6.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초씩 정확</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -13605,6 +13934,9 @@
       </rPr>
       <t xml:space="preserve">재시도 테스트 등 추가</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">여러 비율 파일 이름 테스트 추가</t>
   </si>
 </sst>
 </file>
@@ -13946,8 +14278,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F47"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -13974,8 +14306,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E23"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -14198,7 +14530,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E30,"완료")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14216,7 +14548,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E30,"대기")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14225,7 +14557,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.827586206896552</v>
+        <v>0.862068965517241</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14237,8 +14569,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C46)</f>
-        <v>45</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C47)</f>
+        <v>46</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14246,7 +14578,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B46,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B47,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -14255,8 +14587,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B22,21)</f>
-        <v>91</v>
+        <f aca="false">INDEX(테스트!B2:B23,22)</f>
+        <v>92</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14264,8 +14596,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C22,21)</f>
-        <v>91</v>
+        <f aca="false">INDEX(테스트!C2:C23,22)</f>
+        <v>92</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14887,9 +15219,11 @@
         <v>83</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F28" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="n">
@@ -14963,7 +15297,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -15857,6 +16191,24 @@
         <v>101</v>
       </c>
       <c r="F46" s="8"/>
+    </row>
+    <row r="47" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="F47" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -15877,7 +16229,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -15891,16 +16243,16 @@
         <v>88</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>140</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15918,7 +16270,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15936,7 +16288,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15954,7 +16306,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15972,7 +16324,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15990,7 +16342,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16008,7 +16360,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16026,7 +16378,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16044,7 +16396,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16062,7 +16414,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16080,7 +16432,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16098,7 +16450,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16116,7 +16468,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16134,7 +16486,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16152,7 +16504,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16170,7 +16522,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16188,7 +16540,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16206,7 +16558,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16224,7 +16576,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16242,7 +16594,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16260,7 +16612,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16278,7 +16630,25 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>252</v>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <f aca="false">IFERROR(C23/B23,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Save the current preview scene as a thumbnail image
- Preview button maps the timeline time back to the original file (speed and
  photos included) and grabs the frame at export size, fit and color
- Works for the rendered preview and for a clip's source shown in the player

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="261">
   <si>
     <r>
       <rPr>
@@ -13434,6 +13434,239 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장면을 이미지로 저장 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">썸네일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미리보기 옆 🖼 버튼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완성 미리보기를 보고 있으면 그 시간이 원본 어느 파일의 몇 초인지 계산</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">속도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 원본을 보고 있으면 그 파일에서 바로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">저화질 미리보기가 아니라 원본에서 내보내기 크기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 맞추기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">색감 그대로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JPG/PNG </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">저장</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 1080×1920 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">저장 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -13937,6 +14170,36 @@
   </si>
   <si>
     <t xml:space="preserve">여러 비율 파일 이름 테스트 추가</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장면 위치 계산</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이미지 저장 테스트 추가</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -14278,8 +14541,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F47"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F48"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -14306,8 +14569,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E24"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -14530,7 +14793,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E30,"완료")</f>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14548,7 +14811,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E30,"대기")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14557,7 +14820,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.862068965517241</v>
+        <v>0.896551724137931</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14569,8 +14832,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C47)</f>
-        <v>46</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C48)</f>
+        <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14578,7 +14841,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B47,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B48,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -14587,8 +14850,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B23,22)</f>
-        <v>92</v>
+        <f aca="false">INDEX(테스트!B2:B24,23)</f>
+        <v>94</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14596,8 +14859,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C23,22)</f>
-        <v>92</v>
+        <f aca="false">INDEX(테스트!C2:C24,23)</f>
+        <v>94</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15239,9 +15502,11 @@
         <v>85</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F29" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="n">
@@ -15297,7 +15562,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -16209,6 +16474,24 @@
         <v>231</v>
       </c>
       <c r="F47" s="8"/>
+    </row>
+    <row r="48" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="F48" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -16229,7 +16512,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -16243,16 +16526,16 @@
         <v>88</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>140</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16270,7 +16553,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16288,7 +16571,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16306,7 +16589,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16324,7 +16607,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16342,7 +16625,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16360,7 +16643,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16378,7 +16661,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16396,7 +16679,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16414,7 +16697,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16432,7 +16715,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16450,7 +16733,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16468,7 +16751,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16486,7 +16769,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16504,7 +16787,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16522,7 +16805,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16540,7 +16823,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16558,7 +16841,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16576,7 +16859,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16594,7 +16877,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16612,7 +16895,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16630,7 +16913,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16648,7 +16931,25 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>256</v>
+        <v>259</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <f aca="false">IFERROR(C24/B24,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Subtitle entrance effects: fade and pop
- SubtitleSettings.animation: none | fade | pop (burned-in subtitles only)
- Written as ASS with the same 384x288 header ffmpeg uses for SRT, so the
  existing force_style sizes and positions are unchanged once the effect ends

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="265">
   <si>
     <r>
       <rPr>
@@ -13667,6 +13667,316 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">자막 등장 효과</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">등장 효과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">없음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스르륵 나타나기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">톡 튀어나오기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(70%→112%→100%, 0.18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). ffmpeg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SRT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 읽을 때 효과 태그를 지워 버려서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, SRT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 읽을 때와 똑같은 머리말</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(384×288)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ASS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일로 만들어 입힘 → 효과가 끝난 뒤 화면은 효과 없을 때와 같음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아래</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가운데</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">위 모두 비교</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 트랙 방식에선 꺼짐</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프레임별 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -14199,6 +14509,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">이미지 저장 테스트 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 등장 효과 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
     </r>
   </si>
 </sst>
@@ -14541,8 +14881,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F49"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -14569,8 +14909,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E25"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -14793,7 +15133,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E30,"완료")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14811,7 +15151,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E30,"대기")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14820,7 +15160,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.896551724137931</v>
+        <v>0.931034482758621</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14832,8 +15172,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C48)</f>
-        <v>47</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C49)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14841,7 +15181,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B48,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B49,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -14850,8 +15190,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B24,23)</f>
-        <v>94</v>
+        <f aca="false">INDEX(테스트!B2:B25,24)</f>
+        <v>96</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14859,8 +15199,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C24,23)</f>
-        <v>94</v>
+        <f aca="false">INDEX(테스트!C2:C25,24)</f>
+        <v>96</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15522,9 +15862,11 @@
         <v>87</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F30" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E30">
@@ -15562,7 +15904,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -16492,6 +16834,24 @@
         <v>234</v>
       </c>
       <c r="F48" s="8"/>
+    </row>
+    <row r="49" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="F49" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -16512,7 +16872,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -16526,16 +16886,16 @@
         <v>88</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>140</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16553,7 +16913,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16571,7 +16931,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16589,7 +16949,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16607,7 +16967,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16625,7 +16985,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16643,7 +17003,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16661,7 +17021,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16679,7 +17039,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16697,7 +17057,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16715,7 +17075,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16733,7 +17093,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16751,7 +17111,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16769,7 +17129,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16787,7 +17147,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16805,7 +17165,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16823,7 +17183,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16841,7 +17201,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16859,7 +17219,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16877,7 +17237,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16895,7 +17255,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16913,7 +17273,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16931,7 +17291,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16949,7 +17309,25 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>260</v>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <f aca="false">IFERROR(C25/B25,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tone-map iPhone HDR video; fix export of projects with no sound
- Detect HLG/PQ sources and convert to BT.709 with zscale + mobius tonemap
  for clips, PiP and saved stills (colors no longer come out washed out)
- Skip loudnorm when there is no audio source at all; it produced NaN on
  pure silence and the export failed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="285">
   <si>
     <r>
       <rPr>
@@ -2358,6 +2358,589 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영상 색 바램 고치기</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰은 기본이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">촬영 → 여행 영상 대부분이 회색으로 바래서 나옴 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과물 오류</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰 사진</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(HEIC) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지원</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">아이폰 사진 기본 형식 — 여행 사진을 그대로 넣을 수 있어야 함</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">폴더 통째로 추가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 날짜순 정렬</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여행 영상은 수십</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">~</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수백 개 — 하나씩 고르기 힘들고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여행 순서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 기본 흐름</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 안전 영역 표시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목 위치 자동 회피</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스는 아래쪽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설명</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">버튼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과 오른쪽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">좋아요 등</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 화면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">UI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 가림 — 자막이 가려지면 안 됨</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설정 템플릿 저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">불러오기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다음 여행에 그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다른 여행도 같은 스타일로 만들 계획 — 음악 빼고 컷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">색감</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기 설정 재사용</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 없이 내보내기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">인스타 앱에서 같은 노래 붙이기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">저작권 음악은 인스타에서 음소거될 수 있음 — 비트 컷은 유지하고 소리만 빼서 앱 음악 기능 사용</t>
+  </si>
+  <si>
     <t xml:space="preserve">날짜</t>
   </si>
   <si>
@@ -13977,6 +14560,646 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 로드맵</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일본 여행 릴스용으로 재정렬</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용 목적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일본 여행 영상 모음 → 릴스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다른 여행에도 재사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 맞춰 우선순위 재설정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">색</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 31 HEIC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 32 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">폴더 추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 33 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 안전 영역</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 34 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설정 템플릿</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 35 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 없이 내보내기</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영상이 회색으로 바램</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰 기본 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR(HLG, BT.2020 10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HEVC) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영상을 넣으면 색이 크게 바램</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">채도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">247→94). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영상마다 전달 특성을 확인해서 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">zscale+tonemap(mobius)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">으로 일반 색으로 변환 — 클립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장면 이미지 저장 모두</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">채도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">211</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 회복</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">속도 부담 약 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12%</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수정 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비교 이미지 확인</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">소리가 하나도 없는 영상 내보내기 실패</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무음 영상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진만 있고 음악이 없으면 음량 자동 맞춤</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(loudnorm)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 완전한 무음에서 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NaN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 내서 내보내기가 실패 → 소리가 없을 땐 음량 맞춤을 건너뜀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. HDR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테스트 중 발견</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -14539,6 +15762,46 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">개 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HDR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">색</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무음 내보내기 테스트 추가</t>
     </r>
   </si>
 </sst>
@@ -14747,7 +16010,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -14791,6 +16054,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEEEEEE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -14881,8 +16152,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F52"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -14895,8 +16166,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F36"/>
   <tableColumns count="6">
     <tableColumn id="1" name="순위"/>
     <tableColumn id="2" name="항목"/>
@@ -14909,8 +16180,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -15123,8 +16394,8 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <f aca="false">COUNTA(로드맵!B2:B30)</f>
-        <v>29</v>
+        <f aca="false">COUNTA(로드맵!B2:B36)</f>
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15132,8 +16403,8 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E30,"완료")</f>
-        <v>27</v>
+        <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15141,8 +16412,8 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E30,"진행 중")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF(로드맵!E2:E36,"진행 중")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15150,8 +16421,8 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E30,"대기")</f>
-        <v>2</v>
+        <f aca="false">COUNTIF(로드맵!E2:E36,"대기")</f>
+        <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15160,7 +16431,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.931034482758621</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15172,8 +16443,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C49)</f>
-        <v>48</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C52)</f>
+        <v>51</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15181,7 +16452,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B49,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B52,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -15190,8 +16461,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B25,24)</f>
-        <v>96</v>
+        <f aca="false">INDEX(테스트!B2:B26,25)</f>
+        <v>98</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15199,8 +16470,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C25,24)</f>
-        <v>96</v>
+        <f aca="false">INDEX(테스트!C2:C26,25)</f>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15261,7 +16532,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -15868,21 +17139,131 @@
         <v>28</v>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="8"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E30">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+  <conditionalFormatting sqref="E2:E36">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"완료"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"진행 중"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"대기"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"수정"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"확인 대기"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15904,7 +17285,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -15917,182 +17298,182 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>101</v>
-      </c>
       <c r="F7" s="8" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16100,16 +17481,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -16118,19 +17499,19 @@
         <v>28</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16138,19 +17519,19 @@
         <v>28</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16158,19 +17539,19 @@
         <v>28</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16178,19 +17559,19 @@
         <v>28</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16198,16 +17579,16 @@
         <v>28</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -16216,19 +17597,19 @@
         <v>28</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16236,19 +17617,19 @@
         <v>28</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16256,19 +17637,19 @@
         <v>28</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16276,19 +17657,19 @@
         <v>28</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16296,19 +17677,19 @@
         <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16316,19 +17697,19 @@
         <v>28</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16336,19 +17717,19 @@
         <v>28</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16356,19 +17737,19 @@
         <v>28</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16376,13 +17757,13 @@
         <v>28</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -16392,19 +17773,19 @@
         <v>28</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16412,19 +17793,19 @@
         <v>28</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16432,19 +17813,19 @@
         <v>28</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16452,19 +17833,19 @@
         <v>28</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16472,19 +17853,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16492,13 +17873,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -16508,19 +17889,19 @@
         <v>28</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16528,19 +17909,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16548,19 +17929,19 @@
         <v>28</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16568,13 +17949,13 @@
         <v>28</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
@@ -16584,19 +17965,19 @@
         <v>28</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16604,13 +17985,13 @@
         <v>28</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>2</v>
@@ -16622,19 +18003,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16642,16 +18023,16 @@
         <v>28</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -16660,16 +18041,16 @@
         <v>28</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -16678,16 +18059,16 @@
         <v>28</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -16696,16 +18077,16 @@
         <v>28</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -16714,16 +18095,16 @@
         <v>28</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -16732,16 +18113,16 @@
         <v>28</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -16750,16 +18131,16 @@
         <v>28</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="F44" s="8"/>
     </row>
@@ -16768,16 +18149,16 @@
         <v>28</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="F45" s="8"/>
     </row>
@@ -16786,16 +18167,16 @@
         <v>28</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="F46" s="8"/>
     </row>
@@ -16804,16 +18185,16 @@
         <v>28</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="F47" s="8"/>
     </row>
@@ -16822,16 +18203,16 @@
         <v>28</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="F48" s="8"/>
     </row>
@@ -16840,18 +18221,72 @@
         <v>28</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="F49" s="8"/>
+    </row>
+    <row r="50" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="F50" s="8"/>
+    </row>
+    <row r="51" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="F51" s="8"/>
+    </row>
+    <row r="52" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F52" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -16872,7 +18307,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -16883,24 +18318,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>50</v>
@@ -16913,7 +18348,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16931,7 +18366,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16949,7 +18384,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16967,7 +18402,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16985,7 +18420,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17003,7 +18438,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17021,7 +18456,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17039,7 +18474,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17057,7 +18492,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17075,7 +18510,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17093,7 +18528,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17111,7 +18546,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17129,7 +18564,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17147,7 +18582,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17165,7 +18600,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17183,7 +18618,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17201,7 +18636,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17219,7 +18654,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17237,7 +18672,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17255,7 +18690,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17273,7 +18708,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17291,7 +18726,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17309,7 +18744,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17327,7 +18762,25 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>264</v>
+        <v>283</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <f aca="false">IFERROR(C26/B26,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Support iPhone HEIC photos; upright thumbnails for rotated photos
- HEIC/HEIF photos are converted once to a cached JPEG (EXIF rotation applied)
  for rendering, PiP, stills and thumbnails; projects keep the original path
- Clip list thumbnails honor EXIF orientation
- Bundle pillow-heif in the Windows build and CI

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="289">
   <si>
     <r>
       <rPr>
@@ -15200,6 +15200,410 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아이폰 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HEIC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 지원</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HEIC/HEIF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진을 추가하면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pillow-heif</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 한 번 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JPG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 바꿔 두고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(EXIF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회전 반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">크기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수정 시각 기준 재사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">렌더링</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">썸네일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장면 저장에 사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프로젝트에는 원본 경로 유지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">함께 고침</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목록 썸네일이 세로 사진</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(EXIF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회전</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 가로로 보여 주던 문제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설치본에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pillow-heif </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">포함</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HEIC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">렌더링 방향 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -15802,6 +16206,27 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">무음 내보내기 테스트 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HEIC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 테스트 추가</t>
     </r>
   </si>
 </sst>
@@ -16010,7 +16435,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -16054,14 +16479,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEEEEEE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -16152,8 +16569,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F52"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F53"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -16180,8 +16597,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E27"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -16404,7 +16821,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16413,7 +16830,7 @@
       </c>
       <c r="B5" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"진행 중")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16431,7 +16848,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.8</v>
+        <v>0.828571428571429</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16443,8 +16860,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C52)</f>
-        <v>51</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C53)</f>
+        <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16452,7 +16869,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B52,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B53,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -16461,8 +16878,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B26,25)</f>
-        <v>98</v>
+        <f aca="false">INDEX(테스트!B2:B27,26)</f>
+        <v>99</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16470,8 +16887,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C26,25)</f>
-        <v>98</v>
+        <f aca="false">INDEX(테스트!C2:C27,26)</f>
+        <v>99</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17173,9 +17590,11 @@
         <v>91</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F32" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="n">
@@ -17251,19 +17670,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E36">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"진행 중"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"대기"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"수정"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"확인 대기"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17285,7 +17704,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -18287,6 +18706,24 @@
         <v>113</v>
       </c>
       <c r="F52" s="8"/>
+    </row>
+    <row r="53" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="F53" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -18307,7 +18744,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -18321,16 +18758,16 @@
         <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>152</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18348,7 +18785,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18366,7 +18803,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18384,7 +18821,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18402,7 +18839,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18420,7 +18857,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18438,7 +18875,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18456,7 +18893,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18474,7 +18911,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18492,7 +18929,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18510,7 +18947,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18528,7 +18965,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18546,7 +18983,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18564,7 +19001,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18582,7 +19019,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18600,7 +19037,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18618,7 +19055,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18636,7 +19073,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18654,7 +19091,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18672,7 +19109,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18690,7 +19127,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18708,7 +19145,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18726,7 +19163,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18744,7 +19181,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18762,7 +19199,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18780,7 +19217,25 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>284</v>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <f aca="false">IFERROR(C27/B27,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a whole folder of clips in shooting order; sort by date
- Folder button scans subfolders for videos/photos (skips hidden files and
  sidecars), shows progress, and adds them sorted by shot time
- Shot time from iPhone creationdate (local tz), creation_time, photo EXIF,
  then file mtime; date shown in the clip list; Date-sort button

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="293">
   <si>
     <r>
       <rPr>
@@ -15604,6 +15604,362 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">폴더 통째로 추가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 날짜순</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">📁 폴더</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">하위 폴더까지 영상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진을 찾아</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">숨김 파일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·.AAE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">등 제외</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 시각순으로 추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일이 많으면 진행 창</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그만 버튼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). 📅 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전체 다시 정렬</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 시각은 아이폰 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">creationdate(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현지 시간대 포함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) → creation_time → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사진 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EXIF(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시간대 있으면 반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일 수정 시각 순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목록에 날짜 표시</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도쿄→사진→오사카→교토 순서 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -16227,6 +16583,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">사진 테스트 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 시각</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">폴더 검색 테스트 추가</t>
     </r>
   </si>
 </sst>
@@ -16569,8 +16955,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F54"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -16597,8 +16983,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E28"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -16821,7 +17207,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16839,7 +17225,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"대기")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16848,7 +17234,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.828571428571429</v>
+        <v>0.857142857142857</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16860,8 +17246,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C53)</f>
-        <v>52</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C54)</f>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16869,7 +17255,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B53,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B54,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -16878,8 +17264,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B27,26)</f>
-        <v>99</v>
+        <f aca="false">INDEX(테스트!B2:B28,27)</f>
+        <v>101</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16887,8 +17273,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C27,26)</f>
-        <v>99</v>
+        <f aca="false">INDEX(테스트!C2:C28,27)</f>
+        <v>101</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17610,9 +17996,11 @@
         <v>93</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F33" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="n">
@@ -17704,7 +18092,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -18724,6 +19112,24 @@
         <v>259</v>
       </c>
       <c r="F53" s="8"/>
+    </row>
+    <row r="54" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="F54" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -18744,7 +19150,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -18758,16 +19164,16 @@
         <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>152</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18785,7 +19191,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18803,7 +19209,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18821,7 +19227,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18839,7 +19245,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18857,7 +19263,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18875,7 +19281,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18893,7 +19299,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18911,7 +19317,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18929,7 +19335,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18947,7 +19353,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18965,7 +19371,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18983,7 +19389,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19001,7 +19407,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19019,7 +19425,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19037,7 +19443,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19055,7 +19461,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19073,7 +19479,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19091,7 +19497,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19109,7 +19515,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19127,7 +19533,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19145,7 +19551,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19163,7 +19569,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19181,7 +19587,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19199,7 +19605,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19217,7 +19623,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19235,7 +19641,25 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>288</v>
+        <v>291</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <f aca="false">IFERROR(C28/B28,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep subtitles, titles and PiP out of the Reels UI on vertical videos
- On 9:16 output, bottom/top/right margins grow to about 22%/12%/13% so the
  Reels caption, header and buttons don't cover them (on by default)
- Preview-only overlay tints the covered areas red

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="296">
   <si>
     <r>
       <rPr>
@@ -15960,6 +15960,437 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 가림 영역 피하기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">표시</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기본 자막 위치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아래 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8%)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">와 오른쪽 아래 작은 화면이 릴스 설명</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">버튼에 가려지는 문제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세로 영상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">높이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">너비 ≥ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.6)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이면 자막</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면 여백을 위 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12%/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아래 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22%/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오른쪽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">13% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이상으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이미 더 크면 그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미리보기 전용 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가림 영역 표시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 붉게 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비교 이미지로 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">남은 점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아래쪽 작은 화면과 아래 자막이 겹칠 수 있음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">위치 설정으로 조정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -16613,6 +17044,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">폴더 검색 테스트 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 안전 영역 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
     </r>
   </si>
 </sst>
@@ -16955,8 +17416,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F55"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -16983,8 +17444,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E29"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -17207,7 +17668,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17225,7 +17686,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"대기")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17234,7 +17695,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.857142857142857</v>
+        <v>0.885714285714286</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17246,8 +17707,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C54)</f>
-        <v>53</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C55)</f>
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17255,7 +17716,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B54,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B55,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -17264,8 +17725,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B28,27)</f>
-        <v>101</v>
+        <f aca="false">INDEX(테스트!B2:B29,28)</f>
+        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17273,8 +17734,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C28,27)</f>
-        <v>101</v>
+        <f aca="false">INDEX(테스트!C2:C29,28)</f>
+        <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18016,9 +18477,11 @@
         <v>95</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F34" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="n">
@@ -18092,7 +18555,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -19130,6 +19593,24 @@
         <v>262</v>
       </c>
       <c r="F54" s="8"/>
+    </row>
+    <row r="55" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F55" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -19150,7 +19631,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -19164,16 +19645,16 @@
         <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>152</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19191,7 +19672,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19209,7 +19690,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19227,7 +19708,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19245,7 +19726,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19263,7 +19744,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19281,7 +19762,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19299,7 +19780,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19317,7 +19798,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19335,7 +19816,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19353,7 +19834,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19371,7 +19852,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19389,7 +19870,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19407,7 +19888,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19425,7 +19906,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19443,7 +19924,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19461,7 +19942,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19479,7 +19960,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19497,7 +19978,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19515,7 +19996,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19533,7 +20014,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19551,7 +20032,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19569,7 +20050,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19587,7 +20068,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19605,7 +20086,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19623,7 +20104,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19641,7 +20122,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19659,7 +20140,25 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <f aca="false">IFERROR(C29/B29,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Settings templates to reuse a trip's style on the next one
- Save current settings (cuts, subtitle/title style, color, export) as a named
  template without clips, PiPs, subtitle/title text or output path; music optional
- Apply from the File menu; keeps the current clips and text, undoable

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="300">
   <si>
     <r>
       <rPr>
@@ -16391,6 +16391,391 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설정 템플릿 저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">적용</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일 메뉴</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지금 설정을 템플릿으로 저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이름 입력</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 포함 여부 선택</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿 적용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿 폴더 열기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작은 화면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 내용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목 내용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">출력 경로는 빼고 저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">적용해도 지금 클립</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자막 내용은 그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실행 취소로 되돌릴 수 있음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">저장 위치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">데이터 폴더</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/templates</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 테스트로 저장→적용→실행 취소 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -17055,6 +17440,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">릴스 안전 영역 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿 테스트 </t>
     </r>
     <r>
       <rPr>
@@ -17416,8 +17831,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F56"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -17444,8 +17859,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E30"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -17668,7 +18083,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17686,7 +18101,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"대기")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17695,7 +18110,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.885714285714286</v>
+        <v>0.914285714285714</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17707,8 +18122,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C55)</f>
-        <v>54</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C56)</f>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17716,7 +18131,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B55,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B56,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -17725,8 +18140,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B29,28)</f>
-        <v>103</v>
+        <f aca="false">INDEX(테스트!B2:B30,29)</f>
+        <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17734,8 +18149,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C29,28)</f>
-        <v>103</v>
+        <f aca="false">INDEX(테스트!C2:C30,29)</f>
+        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18497,9 +18912,11 @@
         <v>97</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F35" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="n">
@@ -18555,7 +18972,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -19611,6 +20028,24 @@
         <v>2</v>
       </c>
       <c r="F55" s="8"/>
+    </row>
+    <row r="56" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="F56" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -19631,7 +20066,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -19645,16 +20080,16 @@
         <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>152</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19672,7 +20107,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19690,7 +20125,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19708,7 +20143,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19726,7 +20161,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19744,7 +20179,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19762,7 +20197,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19780,7 +20215,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19798,7 +20233,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19816,7 +20251,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19834,7 +20269,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19852,7 +20287,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19870,7 +20305,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19888,7 +20323,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19906,7 +20341,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19924,7 +20359,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19942,7 +20377,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19960,7 +20395,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19978,7 +20413,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19996,7 +20431,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20014,7 +20449,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20032,7 +20467,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20050,7 +20485,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20068,7 +20503,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20086,7 +20521,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20104,7 +20539,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20122,7 +20557,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20140,7 +20575,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20158,7 +20593,25 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>295</v>
+        <v>298</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <f aca="false">IFERROR(C30/B30,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Option to export without the music track, keeping the beat cuts
- 'Include music' checkbox; when off the cut plan is unchanged and the music
  input is dropped, so the song can be added in the Instagram app instead
- Done dialog says which song and start time to pick in the app

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="303">
   <si>
     <r>
       <rPr>
@@ -16776,6 +16776,248 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">음악 없이 내보내기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내보내기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 넣기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 끄면 비트에 맞춘 컷 계획은 그대로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 트랙만 빼고 만듦</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 창에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">인스타 앱에서 이 노래를 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초부터</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안내</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원본 소리도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이면 완전 무음 영상이 되는데</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">앞서 고친 무음 내보내기 덕분에 정상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(8.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, -91dB) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -17490,6 +17732,9 @@
       </rPr>
       <t xml:space="preserve">개 추가</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">음악 없이 내보내기 테스트 추가</t>
   </si>
 </sst>
 </file>
@@ -17831,8 +18076,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F57"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -17859,8 +18104,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E31"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -18083,7 +18328,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18101,7 +18346,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E36,"대기")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18110,7 +18355,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.914285714285714</v>
+        <v>0.942857142857143</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18122,8 +18367,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C56)</f>
-        <v>55</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C57)</f>
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18131,7 +18376,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B56,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B57,"사용자 제보")</f>
         <v>4</v>
       </c>
     </row>
@@ -18140,8 +18385,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B30,29)</f>
-        <v>105</v>
+        <f aca="false">INDEX(테스트!B2:B31,30)</f>
+        <v>106</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18149,8 +18394,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C30,29)</f>
-        <v>105</v>
+        <f aca="false">INDEX(테스트!C2:C31,30)</f>
+        <v>106</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18932,9 +19177,11 @@
         <v>99</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F36" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E36">
@@ -18972,7 +19219,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -20046,6 +20293,24 @@
         <v>267</v>
       </c>
       <c r="F56" s="8"/>
+    </row>
+    <row r="57" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F57" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -20066,7 +20331,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -20080,16 +20345,16 @@
         <v>100</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>152</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20107,7 +20372,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20125,7 +20390,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20143,7 +20408,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20161,7 +20426,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20179,7 +20444,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20197,7 +20462,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20215,7 +20480,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20233,7 +20498,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20251,7 +20516,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20269,7 +20534,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20287,7 +20552,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20305,7 +20570,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20323,7 +20588,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20341,7 +20606,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20359,7 +20624,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20377,7 +20642,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20395,7 +20660,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20413,7 +20678,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20431,7 +20696,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20449,7 +20714,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20467,7 +20732,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20485,7 +20750,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20503,7 +20768,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20521,7 +20786,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20539,7 +20804,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20557,7 +20822,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20575,7 +20840,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20593,7 +20858,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20611,7 +20876,25 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>299</v>
+        <v>301</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <f aca="false">IFERROR(C31/B31,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ask when undated clips were shot; editable shot time per clip
- Clips whose time came only from the file mtime are listed in a dialog with
  thumbnails to set the real date (bulk date keeps time-of-day order) or skip
- Shot time field in the clip editor; guessed times marked with a warning

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="318">
   <si>
     <r>
       <rPr>
@@ -2941,6 +2941,223 @@
     <t xml:space="preserve">저작권 음악은 인스타에서 음소거될 수 있음 — 비트 컷은 유지하고 소리만 빼서 앱 음악 기능 사용</t>
   </si>
   <si>
+    <t xml:space="preserve">찍은 날짜 정보가 없으면 물어보기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자 제안 — 메신저로 받은 사진은 날짜가 지워져 날짜순이 틀어짐</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">recap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 특히 중요</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립마다 날짜 도장 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">예</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 2026.03.14)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">recap </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스의 대표 연출 — 언제 장면인지 보여 줌</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월별 제목 자동 만들기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(JANUARY, FEBRUARY …)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년치 영상의 구간 나누기를 손으로 하면 오래 걸림</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">폴더 추가 때 날짜 범위로 고르기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">예</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">카메라 앨범 폴더엔 다른 해 사진도 섞여 있음</t>
+  </si>
+  <si>
     <t xml:space="preserve">날짜</t>
   </si>
   <si>
@@ -17018,6 +17235,484 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 정보 없을 때 물어보기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ 2026 recap </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 계획</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 시간 정보가 없을 때 언제 찍었는지 물어보면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">?" + "2026 recap </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스도 만들 것</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" → 7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 로드맵</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 날짜 묻기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 37 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 도장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 38 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월별 제목 자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 39 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 범위로 골라 추가</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">반영</t>
+  </si>
+  <si>
+    <t xml:space="preserve">찍은 날짜 묻기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립을 추가할 때 촬영 시각 정보가 없어 파일 시각으로 추정한 클립만 모아 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 날짜 정하기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">창</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">썸네일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜시간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모두 이 날짜로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">분은 두고 날짜만 바꿔 같은 날 순서 유지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건너뛰기 가능</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 편집에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 시각</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">칸 추가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추정 시각은 목록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">편집 칸에 ⚠ 표시</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 테스트</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -17735,6 +18430,9 @@
   </si>
   <si>
     <t xml:space="preserve">음악 없이 내보내기 테스트 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">찍은 시각 출처 검사 추가</t>
   </si>
 </sst>
 </file>
@@ -18076,8 +18774,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F59"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -18090,8 +18788,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F40"/>
   <tableColumns count="6">
     <tableColumn id="1" name="순위"/>
     <tableColumn id="2" name="항목"/>
@@ -18104,8 +18802,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E32"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -18318,8 +19016,8 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <f aca="false">COUNTA(로드맵!B2:B36)</f>
-        <v>35</v>
+        <f aca="false">COUNTA(로드맵!B2:B40)</f>
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18327,8 +19025,8 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E36,"완료")</f>
-        <v>33</v>
+        <f aca="false">COUNTIF(로드맵!E2:E40,"완료")</f>
+        <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18336,7 +19034,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E36,"진행 중")</f>
+        <f aca="false">COUNTIF(로드맵!E2:E40,"진행 중")</f>
         <v>0</v>
       </c>
     </row>
@@ -18345,8 +19043,8 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E36,"대기")</f>
-        <v>2</v>
+        <f aca="false">COUNTIF(로드맵!E2:E40,"대기")</f>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18355,7 +19053,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.942857142857143</v>
+        <v>0.871794871794872</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18367,8 +19065,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C57)</f>
-        <v>56</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C59)</f>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18376,8 +19074,8 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B57,"사용자 제보")</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('개발 기록'!B2:B59,"사용자 제보")</f>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18385,7 +19083,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B31,30)</f>
+        <f aca="false">INDEX(테스트!B2:B32,31)</f>
         <v>106</v>
       </c>
     </row>
@@ -18394,7 +19092,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C31,30)</f>
+        <f aca="false">INDEX(테스트!C2:C32,31)</f>
         <v>106</v>
       </c>
     </row>
@@ -18456,7 +19154,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -19183,8 +19881,82 @@
         <v>28</v>
       </c>
     </row>
+    <row r="37" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F40" s="8"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E36">
+  <conditionalFormatting sqref="E2:E40">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
@@ -19219,7 +19991,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -19232,182 +20004,182 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19415,16 +20187,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -19433,19 +20205,19 @@
         <v>28</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19453,19 +20225,19 @@
         <v>28</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19473,19 +20245,19 @@
         <v>28</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19493,19 +20265,19 @@
         <v>28</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19513,16 +20285,16 @@
         <v>28</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -19531,19 +20303,19 @@
         <v>28</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19551,19 +20323,19 @@
         <v>28</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19571,19 +20343,19 @@
         <v>28</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19591,19 +20363,19 @@
         <v>28</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19611,19 +20383,19 @@
         <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19631,19 +20403,19 @@
         <v>28</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19651,19 +20423,19 @@
         <v>28</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19671,19 +20443,19 @@
         <v>28</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19691,13 +20463,13 @@
         <v>28</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -19707,19 +20479,19 @@
         <v>28</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19727,19 +20499,19 @@
         <v>28</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19747,19 +20519,19 @@
         <v>28</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19767,19 +20539,19 @@
         <v>28</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19787,19 +20559,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19807,13 +20579,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -19823,19 +20595,19 @@
         <v>28</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19843,19 +20615,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19863,19 +20635,19 @@
         <v>28</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19883,13 +20655,13 @@
         <v>28</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
@@ -19899,19 +20671,19 @@
         <v>28</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19919,13 +20691,13 @@
         <v>28</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>2</v>
@@ -19937,19 +20709,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19957,16 +20729,16 @@
         <v>28</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -19975,16 +20747,16 @@
         <v>28</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -19993,16 +20765,16 @@
         <v>28</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -20011,16 +20783,16 @@
         <v>28</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -20029,16 +20801,16 @@
         <v>28</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -20047,16 +20819,16 @@
         <v>28</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -20065,16 +20837,16 @@
         <v>28</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="F44" s="8"/>
     </row>
@@ -20083,16 +20855,16 @@
         <v>28</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="F45" s="8"/>
     </row>
@@ -20101,16 +20873,16 @@
         <v>28</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F46" s="8"/>
     </row>
@@ -20119,16 +20891,16 @@
         <v>28</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="F47" s="8"/>
     </row>
@@ -20137,16 +20909,16 @@
         <v>28</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="F48" s="8"/>
     </row>
@@ -20155,16 +20927,16 @@
         <v>28</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F49" s="8"/>
     </row>
@@ -20173,16 +20945,16 @@
         <v>28</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="F50" s="8"/>
     </row>
@@ -20191,16 +20963,16 @@
         <v>28</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="F51" s="8"/>
     </row>
@@ -20209,16 +20981,16 @@
         <v>28</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F52" s="8"/>
     </row>
@@ -20227,16 +20999,16 @@
         <v>28</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="F53" s="8"/>
     </row>
@@ -20245,16 +21017,16 @@
         <v>28</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="F54" s="8"/>
     </row>
@@ -20263,13 +21035,13 @@
         <v>28</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>2</v>
@@ -20281,16 +21053,16 @@
         <v>28</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="F56" s="8"/>
     </row>
@@ -20299,18 +21071,54 @@
         <v>28</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F57" s="8"/>
+    </row>
+    <row r="58" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="F58" s="8"/>
+    </row>
+    <row r="59" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="F59" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -20331,7 +21139,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -20342,24 +21150,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>50</v>
@@ -20372,7 +21180,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20390,7 +21198,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20408,7 +21216,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20426,7 +21234,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20444,7 +21252,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20462,7 +21270,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20480,7 +21288,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20498,7 +21306,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20516,7 +21324,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20534,7 +21342,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20552,7 +21360,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20570,7 +21378,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20588,7 +21396,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20606,7 +21414,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20624,7 +21432,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20642,7 +21450,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20660,7 +21468,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20678,7 +21486,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20696,7 +21504,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20714,7 +21522,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20732,7 +21540,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20750,7 +21558,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20768,7 +21576,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20786,7 +21594,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20804,7 +21612,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20822,7 +21630,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20840,7 +21648,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20858,7 +21666,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20876,7 +21684,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20894,7 +21702,25 @@
         <v>1</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>302</v>
+        <v>316</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <f aca="false">IFERROR(C32/B32,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Date stamp overlay showing each clip's shot date
- Film-camera style (orange digits, '26 3 14) or plain white in five formats,
  any corner, avoiding the Reels UI area
- Events follow the frame-rounded segment timing; repeated dates merge,
  clips without a date show nothing

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="322">
   <si>
     <r>
       <rPr>
@@ -17713,6 +17713,259 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">날짜 도장</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목 탭 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 도장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">필름 카메라</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">주황 숫자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, '26 3 14) / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">깔끔한 흰 글자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">형식 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">네 구석 위치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">렌더링과 같은 프레임 단위로 조각마다 그 클립의 찍은 날짜를 넣고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같은 날짜가 이어지면 하나로 합침</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 모르는 클립은 표시 안 함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴스 가림 영역도 피함</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -18433,6 +18686,9 @@
   </si>
   <si>
     <t xml:space="preserve">찍은 시각 출처 검사 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">날짜 도장 테스트 추가</t>
   </si>
 </sst>
 </file>
@@ -18774,8 +19030,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F60"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -18802,8 +19058,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -19026,7 +19282,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E40,"완료")</f>
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19044,7 +19300,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E40,"대기")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19053,7 +19309,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.871794871794872</v>
+        <v>0.897435897435898</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19065,8 +19321,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C59)</f>
-        <v>58</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C60)</f>
+        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19074,7 +19330,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B59,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B60,"사용자 제보")</f>
         <v>5</v>
       </c>
     </row>
@@ -19083,8 +19339,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B32,31)</f>
-        <v>106</v>
+        <f aca="false">INDEX(테스트!B2:B33,32)</f>
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19092,8 +19348,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C32,31)</f>
-        <v>106</v>
+        <f aca="false">INDEX(테스트!C2:C33,32)</f>
+        <v>107</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19915,9 +20171,11 @@
         <v>103</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F38" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="n">
@@ -19991,7 +20249,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21119,6 +21377,24 @@
         <v>283</v>
       </c>
       <c r="F59" s="8"/>
+    </row>
+    <row r="60" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="F60" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -21139,7 +21415,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21153,16 +21429,16 @@
         <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21180,7 +21456,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21198,7 +21474,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21216,7 +21492,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21234,7 +21510,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21252,7 +21528,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21270,7 +21546,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21288,7 +21564,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21306,7 +21582,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21324,7 +21600,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21342,7 +21618,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21360,7 +21636,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21378,7 +21654,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21396,7 +21672,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21414,7 +21690,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21432,7 +21708,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21450,7 +21726,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21468,7 +21744,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21486,7 +21762,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21504,7 +21780,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21522,7 +21798,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21540,7 +21816,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21558,7 +21834,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21576,7 +21852,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21594,7 +21870,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21612,7 +21888,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21630,7 +21906,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21648,7 +21924,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21666,7 +21942,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21684,7 +21960,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21702,7 +21978,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21720,7 +21996,25 @@
         <v>1</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>317</v>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <f aca="false">IFERROR(C33/B33,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Automatic month titles from clip shot dates
- Titles tab button adds JANUARY/JAN/1월/01 titles where the month changes
  in the finished timeline; shortened if the next month starts sooner
- Choose to replace or keep existing titles

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="325">
   <si>
     <r>
       <rPr>
@@ -17966,6 +17966,248 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">월별 제목 자동</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제목 탭 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"📅 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월별 제목 자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"(JANUARY/JAN/1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/01): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완성 영상 조각을 따라가며 찍은 날짜의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 바뀌는 순간에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 제목</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다음 달이 더 빨리 오면 거기서 끝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 없는 클립은 건너뜀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기존 제목은 지우고 넣기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같이 두기 선택</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개발 중 버튼 기능이 자막 패널에 잘못 붙은 것을 화면 테스트에서 발견해 바로잡음</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -18689,6 +18931,9 @@
   </si>
   <si>
     <t xml:space="preserve">날짜 도장 테스트 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">월별 제목 테스트 추가</t>
   </si>
 </sst>
 </file>
@@ -19030,8 +19275,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F61"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -19058,8 +19303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E34"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -19282,7 +19527,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E40,"완료")</f>
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19300,7 +19545,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E40,"대기")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19309,7 +19554,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.897435897435898</v>
+        <v>0.923076923076923</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19321,8 +19566,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C60)</f>
-        <v>59</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C61)</f>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19330,7 +19575,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B60,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B61,"사용자 제보")</f>
         <v>5</v>
       </c>
     </row>
@@ -19339,8 +19584,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B33,32)</f>
-        <v>107</v>
+        <f aca="false">INDEX(테스트!B2:B34,33)</f>
+        <v>108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19348,8 +19593,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C33,32)</f>
-        <v>107</v>
+        <f aca="false">INDEX(테스트!C2:C34,33)</f>
+        <v>108</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20191,9 +20436,11 @@
         <v>105</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F39" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="n">
@@ -20249,7 +20496,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21395,6 +21642,24 @@
         <v>286</v>
       </c>
       <c r="F60" s="8"/>
+    </row>
+    <row r="61" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F61" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -21415,7 +21680,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21429,16 +21694,16 @@
         <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21456,7 +21721,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21474,7 +21739,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21492,7 +21757,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21510,7 +21775,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21528,7 +21793,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21546,7 +21811,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21564,7 +21829,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21582,7 +21847,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21600,7 +21865,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21618,7 +21883,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21636,7 +21901,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21654,7 +21919,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21672,7 +21937,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21690,7 +21955,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21708,7 +21973,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21726,7 +21991,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21744,7 +22009,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21762,7 +22027,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21780,7 +22045,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21798,7 +22063,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21816,7 +22081,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21834,7 +22099,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21852,7 +22117,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21870,7 +22135,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21888,7 +22153,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21906,7 +22171,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21924,7 +22189,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21942,7 +22207,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21960,7 +22225,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21978,7 +22243,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21996,7 +22261,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22014,7 +22279,25 @@
         <v>1</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <f aca="false">IFERROR(C34/B34,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Filter a folder by shot-date range when adding (e.g. only 2026)
- Folder add dialog shows the file count and an optional date range with
  this-year/last-year shortcuts; dated files outside are skipped, undated
  files are kept and asked about

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="329">
   <si>
     <r>
       <rPr>
@@ -18208,6 +18208,240 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">폴더 추가 때 날짜 범위로 고르기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">폴더를 고르면 찾은 개수와 함께 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찍은 날짜로 고르기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시작</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">~</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">끝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">올해</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작년 버튼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">창</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜가 확실한 파일만 범위로 거르고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 정보 없는 파일은 넣은 뒤 언제 찍었는지 물어봄</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">뺀 개수 안내</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 2025/2027 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파일 제외</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 없는 파일은 질문 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -18934,6 +19168,9 @@
   </si>
   <si>
     <t xml:space="preserve">월별 제목 테스트 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화면 테스트로 날짜 범위 확인</t>
   </si>
 </sst>
 </file>
@@ -19275,8 +19512,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F62"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -19303,8 +19540,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E35"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -19527,7 +19764,7 @@
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E40,"완료")</f>
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19545,7 +19782,7 @@
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF(로드맵!E2:E40,"대기")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19554,7 +19791,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.923076923076923</v>
+        <v>0.948717948717949</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19566,8 +19803,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C61)</f>
-        <v>60</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C62)</f>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19575,7 +19812,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B61,"사용자 제보")</f>
+        <f aca="false">COUNTIF('개발 기록'!B2:B62,"사용자 제보")</f>
         <v>5</v>
       </c>
     </row>
@@ -19584,7 +19821,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B34,33)</f>
+        <f aca="false">INDEX(테스트!B2:B35,34)</f>
         <v>108</v>
       </c>
     </row>
@@ -19593,7 +19830,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C34,33)</f>
+        <f aca="false">INDEX(테스트!C2:C35,34)</f>
         <v>108</v>
       </c>
     </row>
@@ -20456,9 +20693,11 @@
         <v>107</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F40" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E40">
@@ -20496,7 +20735,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21660,6 +21899,24 @@
         <v>2</v>
       </c>
       <c r="F61" s="8"/>
+    </row>
+    <row r="62" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="F62" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -21680,7 +21937,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21694,16 +21951,16 @@
         <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>160</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21721,7 +21978,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21739,7 +21996,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21757,7 +22014,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21775,7 +22032,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21793,7 +22050,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21811,7 +22068,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21829,7 +22086,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21847,7 +22104,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21865,7 +22122,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21883,7 +22140,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21901,7 +22158,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21919,7 +22176,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21937,7 +22194,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21955,7 +22212,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21973,7 +22230,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21991,7 +22248,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22009,7 +22266,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22027,7 +22284,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22045,7 +22302,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22063,7 +22320,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22081,7 +22338,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22099,7 +22356,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22117,7 +22374,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22135,7 +22392,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22153,7 +22410,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22171,7 +22428,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22189,7 +22446,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22207,7 +22464,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22225,7 +22482,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22243,7 +22500,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22261,7 +22518,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22279,7 +22536,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22297,7 +22554,25 @@
         <v>1</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>324</v>
+        <v>327</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <f aca="false">IFERROR(C35/B35,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Per-clip beat count for beat-synced cuts
- Clip.cut_beats (0 = global setting): each clip stays for its own number of
  beats before the next clip, in clip order
- Applies with 'clip count x cut length' (random order included) and the
  alternating order; other orders keep the global plan with a hint
- Clip editor control, list badge, and length info in the music tab

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="337">
   <si>
     <r>
       <rPr>
@@ -3158,6 +3158,95 @@
     <t xml:space="preserve">카메라 앨범 폴더엔 다른 해 사진도 섞여 있음</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립마다 비트 수 따로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트 …</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자 요청 — 어떤 장면은 짧게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">어떤 장면은 길게</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">날짜</t>
   </si>
   <si>
@@ -18442,6 +18531,416 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">클립마다 비트 수 다르게</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">어떤 영상은 비트 한 번 만에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">어떤 영상은 비트 두 번 뒤에 다음 영상으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요청</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">클립마다 비트 수 따로</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 편집 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트 맞춤 컷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 탭 설정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)/1/2/3/4/8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클립 순서대로 각자 정한 비트만큼 지나서 다음 컷 — 클립 개수 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">컷 길이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무작위 순서도 섞인 순서대로 반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">와 파일 번갈아</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반복</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 적용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그 밖의 방식에선 전체 설정 사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 탭에 안내</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목록에 ♪</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트 표시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 탭 완성 길이 계산에 반영</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· 1+2+4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= 3.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초 확인</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -19171,6 +19670,9 @@
   </si>
   <si>
     <t xml:space="preserve">화면 테스트로 날짜 범위 확인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">클립별 비트 수 테스트 추가</t>
   </si>
 </sst>
 </file>
@@ -19512,8 +20014,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F62"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F64"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -19526,8 +20028,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F41"/>
   <tableColumns count="6">
     <tableColumn id="1" name="순위"/>
     <tableColumn id="2" name="항목"/>
@@ -19540,8 +20042,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E36"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -19754,8 +20256,8 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <f aca="false">COUNTA(로드맵!B2:B40)</f>
-        <v>39</v>
+        <f aca="false">COUNTA(로드맵!B2:B41)</f>
+        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19763,8 +20265,8 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E40,"완료")</f>
-        <v>37</v>
+        <f aca="false">COUNTIF(로드맵!E2:E41,"완료")</f>
+        <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19772,7 +20274,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E40,"진행 중")</f>
+        <f aca="false">COUNTIF(로드맵!E2:E41,"진행 중")</f>
         <v>0</v>
       </c>
     </row>
@@ -19781,7 +20283,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E40,"대기")</f>
+        <f aca="false">COUNTIF(로드맵!E2:E41,"대기")</f>
         <v>2</v>
       </c>
     </row>
@@ -19791,7 +20293,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.948717948717949</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19803,8 +20305,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C62)</f>
-        <v>61</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C64)</f>
+        <v>63</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19812,8 +20314,8 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B62,"사용자 제보")</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('개발 기록'!B2:B64,"사용자 제보")</f>
+        <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19821,8 +20323,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B35,34)</f>
-        <v>108</v>
+        <f aca="false">INDEX(테스트!B2:B36,35)</f>
+        <v>109</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19830,8 +20332,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C35,34)</f>
-        <v>108</v>
+        <f aca="false">INDEX(테스트!C2:C36,35)</f>
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19892,7 +20394,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -20699,8 +21201,28 @@
         <v>28</v>
       </c>
     </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E40">
+  <conditionalFormatting sqref="E2:E41">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
@@ -20735,7 +21257,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -20748,182 +21270,182 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>122</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20931,16 +21453,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -20949,19 +21471,19 @@
         <v>28</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20969,19 +21491,19 @@
         <v>28</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20989,19 +21511,19 @@
         <v>28</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21009,19 +21531,19 @@
         <v>28</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21029,16 +21551,16 @@
         <v>28</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -21047,19 +21569,19 @@
         <v>28</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21067,19 +21589,19 @@
         <v>28</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21087,19 +21609,19 @@
         <v>28</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21107,19 +21629,19 @@
         <v>28</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21127,19 +21649,19 @@
         <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21147,19 +21669,19 @@
         <v>28</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21167,19 +21689,19 @@
         <v>28</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C22" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>179</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21187,19 +21709,19 @@
         <v>28</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21207,13 +21729,13 @@
         <v>28</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -21223,19 +21745,19 @@
         <v>28</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21243,19 +21765,19 @@
         <v>28</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21263,19 +21785,19 @@
         <v>28</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21283,19 +21805,19 @@
         <v>28</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21303,19 +21825,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21323,13 +21845,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -21339,19 +21861,19 @@
         <v>28</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21359,19 +21881,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21379,19 +21901,19 @@
         <v>28</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D33" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="F33" s="8" t="s">
         <v>212</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21399,13 +21921,13 @@
         <v>28</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
@@ -21415,19 +21937,19 @@
         <v>28</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21435,13 +21957,13 @@
         <v>28</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>2</v>
@@ -21453,19 +21975,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21473,16 +21995,16 @@
         <v>28</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -21491,16 +22013,16 @@
         <v>28</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -21509,16 +22031,16 @@
         <v>28</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -21527,16 +22049,16 @@
         <v>28</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -21545,16 +22067,16 @@
         <v>28</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -21563,16 +22085,16 @@
         <v>28</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -21581,16 +22103,16 @@
         <v>28</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F44" s="8"/>
     </row>
@@ -21599,16 +22121,16 @@
         <v>28</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F45" s="8"/>
     </row>
@@ -21617,16 +22139,16 @@
         <v>28</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F46" s="8"/>
     </row>
@@ -21635,16 +22157,16 @@
         <v>28</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F47" s="8"/>
     </row>
@@ -21653,16 +22175,16 @@
         <v>28</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F48" s="8"/>
     </row>
@@ -21671,16 +22193,16 @@
         <v>28</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F49" s="8"/>
     </row>
@@ -21689,16 +22211,16 @@
         <v>28</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F50" s="8"/>
     </row>
@@ -21707,16 +22229,16 @@
         <v>28</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F51" s="8"/>
     </row>
@@ -21725,16 +22247,16 @@
         <v>28</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F52" s="8"/>
     </row>
@@ -21743,16 +22265,16 @@
         <v>28</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F53" s="8"/>
     </row>
@@ -21761,16 +22283,16 @@
         <v>28</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F54" s="8"/>
     </row>
@@ -21779,13 +22301,13 @@
         <v>28</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>2</v>
@@ -21797,16 +22319,16 @@
         <v>28</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F56" s="8"/>
     </row>
@@ -21815,13 +22337,13 @@
         <v>28</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>2</v>
@@ -21833,16 +22355,16 @@
         <v>28</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F58" s="8"/>
     </row>
@@ -21851,16 +22373,16 @@
         <v>28</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F59" s="8"/>
     </row>
@@ -21869,16 +22391,16 @@
         <v>28</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="F60" s="8"/>
     </row>
@@ -21887,13 +22409,13 @@
         <v>28</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>2</v>
@@ -21905,18 +22427,54 @@
         <v>28</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F62" s="8"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="F63" s="8"/>
+    </row>
+    <row r="64" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="F64" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -21937,7 +22495,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21948,24 +22506,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>50</v>
@@ -21978,7 +22536,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21996,7 +22554,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22014,7 +22572,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22032,7 +22590,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22050,7 +22608,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22068,7 +22626,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22086,7 +22644,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22104,7 +22662,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22122,7 +22680,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22140,7 +22698,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22158,7 +22716,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22176,7 +22734,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22194,7 +22752,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22212,7 +22770,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22230,7 +22788,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22248,7 +22806,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22266,7 +22824,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22284,7 +22842,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22302,7 +22860,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22320,7 +22878,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22338,7 +22896,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22356,7 +22914,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22374,7 +22932,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22392,7 +22950,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22410,7 +22968,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22428,7 +22986,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22446,7 +23004,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22464,7 +23022,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22482,7 +23040,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22500,7 +23058,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22518,7 +23076,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22536,7 +23094,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22554,7 +23112,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22572,7 +23130,25 @@
         <v>1</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>328</v>
+        <v>335</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="D36" s="10" t="n">
+        <f aca="false">IFERROR(C36/B36,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Listening history from Google Takeout: top songs of a year
- Read the Takeout zip or watch-history JSON locally; YouTube Music plays by
  default, optionally music-looking YouTube videos; ads, removed videos and
  searches skipped; Korean/English/Japanese title phrasing cleaned up
- Dialog ranks songs by play count per year with search, CSV export, open in
  YouTube, and a one-click download into the music slot
- Step-by-step Takeout guide shown beside the list

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3uaKasMbHBDWfZhRwy6Ns
</commit_message>
<xml_diff>
--- a/video/DEVLOG.xlsx
+++ b/video/DEVLOG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="346">
   <si>
     <r>
       <rPr>
@@ -3247,6 +3247,79 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내가 들은 노래 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구글 테이크아웃 시청 기록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자 요청 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026 recap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 그해 많이 들은 노래 쓰기</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-29</t>
+  </si>
+  <si>
     <t xml:space="preserve">날짜</t>
   </si>
   <si>
@@ -18941,6 +19014,784 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브 좋아요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그해 들은 노래 목록</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브 연결해서 좋아요한 노래 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해당 연도에 들은 노래 리스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 시청 기록을 주지 않아 구글 테이크아웃 시청 기록으로 만들기로 함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테이크아웃 하는 법도 옆에 적어 놔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요청</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내가 들은 노래 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테이크아웃</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">음악 탭 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"📊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내가 들은 노래</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">": </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테이크아웃 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">zip </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">또는 시청 기록 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JSON</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 열면 연도별 많이 들은 순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재생 수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같으면 최근 순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. YouTube Music </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기록 기본</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, "YouTube</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 본 뮤직비디오도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공식 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MV·- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">주제 채널 등</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선택</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">광고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">삭제된 영상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">검색 기록 제외</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">한국어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">영어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일본어 제목 문구 정리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">찾기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">유튜브에서 듣기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, CSV </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">저장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고르면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">mp3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">받기→음악 등록 흐름으로 연결</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">창 오른쪽에 테이크아웃 받는 법</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(HTML </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아닌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JSON </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고르기 강조</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). HTML</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 받았으면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JSON</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">으로 다시 받으라고 안내</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가짜 기록 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">163</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개로 화면 테스트</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">테스트 수</t>
   </si>
   <si>
@@ -19673,6 +20524,36 @@
   </si>
   <si>
     <t xml:space="preserve">클립별 비트 수 테스트 추가</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테이크아웃 기록 테스트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 추가</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -20014,8 +20895,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Log" displayName="Log" ref="A1:F66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F66"/>
   <tableColumns count="6">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="구분"/>
@@ -20028,8 +20909,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Roadmap" displayName="Roadmap" ref="A1:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F42"/>
   <tableColumns count="6">
     <tableColumn id="1" name="순위"/>
     <tableColumn id="2" name="항목"/>
@@ -20042,8 +20923,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tests" displayName="Tests" ref="A1:E37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E37"/>
   <tableColumns count="5">
     <tableColumn id="1" name="날짜"/>
     <tableColumn id="2" name="테스트 수"/>
@@ -20256,8 +21137,8 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <f aca="false">COUNTA(로드맵!B2:B41)</f>
-        <v>40</v>
+        <f aca="false">COUNTA(로드맵!B2:B42)</f>
+        <v>41</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20265,8 +21146,8 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E41,"완료")</f>
-        <v>38</v>
+        <f aca="false">COUNTIF(로드맵!E2:E42,"완료")</f>
+        <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20274,7 +21155,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E41,"진행 중")</f>
+        <f aca="false">COUNTIF(로드맵!E2:E42,"진행 중")</f>
         <v>0</v>
       </c>
     </row>
@@ -20283,7 +21164,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <f aca="false">COUNTIF(로드맵!E2:E41,"대기")</f>
+        <f aca="false">COUNTIF(로드맵!E2:E42,"대기")</f>
         <v>2</v>
       </c>
     </row>
@@ -20293,7 +21174,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">IFERROR(B4/B3,0)</f>
-        <v>0.95</v>
+        <v>0.951219512195122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20305,8 +21186,8 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <f aca="false">COUNTA('개발 기록'!C2:C64)</f>
-        <v>63</v>
+        <f aca="false">COUNTA('개발 기록'!C2:C66)</f>
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20314,8 +21195,8 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <f aca="false">COUNTIF('개발 기록'!B2:B64,"사용자 제보")</f>
-        <v>6</v>
+        <f aca="false">COUNTIF('개발 기록'!B2:B66,"사용자 제보")</f>
+        <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20323,8 +21204,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <f aca="false">INDEX(테스트!B2:B36,35)</f>
-        <v>109</v>
+        <f aca="false">INDEX(테스트!B2:B37,36)</f>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20332,8 +21213,8 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <f aca="false">INDEX(테스트!C2:C36,35)</f>
-        <v>109</v>
+        <f aca="false">INDEX(테스트!C2:C37,36)</f>
+        <v>112</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20394,7 +21275,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -21221,8 +22102,28 @@
         <v>28</v>
       </c>
     </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E41">
+  <conditionalFormatting sqref="E2:E42">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"완료"</formula>
     </cfRule>
@@ -21257,7 +22158,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -21270,182 +22171,182 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D4" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>125</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21453,16 +22354,16 @@
         <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -21471,19 +22372,19 @@
         <v>28</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21491,19 +22392,19 @@
         <v>28</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21511,19 +22412,19 @@
         <v>28</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21531,19 +22432,19 @@
         <v>28</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21551,16 +22452,16 @@
         <v>28</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -21569,19 +22470,19 @@
         <v>28</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21589,19 +22490,19 @@
         <v>28</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21609,19 +22510,19 @@
         <v>28</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21629,19 +22530,19 @@
         <v>28</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21649,19 +22550,19 @@
         <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21669,19 +22570,19 @@
         <v>28</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21689,19 +22590,19 @@
         <v>28</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D22" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>182</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21709,19 +22610,19 @@
         <v>28</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21729,13 +22630,13 @@
         <v>28</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -21745,19 +22646,19 @@
         <v>28</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21765,19 +22666,19 @@
         <v>28</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21785,19 +22686,19 @@
         <v>28</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21805,19 +22706,19 @@
         <v>28</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21825,19 +22726,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21845,13 +22746,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -21861,19 +22762,19 @@
         <v>28</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21881,19 +22782,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21901,19 +22802,19 @@
         <v>28</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21921,13 +22822,13 @@
         <v>28</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
@@ -21937,19 +22838,19 @@
         <v>28</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>2</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21957,13 +22858,13 @@
         <v>28</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>2</v>
@@ -21975,19 +22876,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21995,16 +22896,16 @@
         <v>28</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -22013,16 +22914,16 @@
         <v>28</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -22031,16 +22932,16 @@
         <v>28</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -22049,16 +22950,16 @@
         <v>28</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -22067,16 +22968,16 @@
         <v>28</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -22085,16 +22986,16 @@
         <v>28</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -22103,16 +23004,16 @@
         <v>28</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F44" s="8"/>
     </row>
@@ -22121,16 +23022,16 @@
         <v>28</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="F45" s="8"/>
     </row>
@@ -22139,16 +23040,16 @@
         <v>28</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F46" s="8"/>
     </row>
@@ -22157,16 +23058,16 @@
         <v>28</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F47" s="8"/>
     </row>
@@ -22175,16 +23076,16 @@
         <v>28</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F48" s="8"/>
     </row>
@@ -22193,16 +23094,16 @@
         <v>28</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F49" s="8"/>
     </row>
@@ -22211,16 +23112,16 @@
         <v>28</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F50" s="8"/>
     </row>
@@ -22229,16 +23130,16 @@
         <v>28</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F51" s="8"/>
     </row>
@@ -22247,16 +23148,16 @@
         <v>28</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F52" s="8"/>
     </row>
@@ -22265,16 +23166,16 @@
         <v>28</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F53" s="8"/>
     </row>
@@ -22283,16 +23184,16 @@
         <v>28</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F54" s="8"/>
     </row>
@@ -22301,13 +23202,13 @@
         <v>28</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>2</v>
@@ -22319,16 +23220,16 @@
         <v>28</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F56" s="8"/>
     </row>
@@ -22337,13 +23238,13 @@
         <v>28</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>2</v>
@@ -22355,16 +23256,16 @@
         <v>28</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F58" s="8"/>
     </row>
@@ -22373,16 +23274,16 @@
         <v>28</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="F59" s="8"/>
     </row>
@@ -22391,16 +23292,16 @@
         <v>28</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="F60" s="8"/>
     </row>
@@ -22409,13 +23310,13 @@
         <v>28</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>2</v>
@@ -22427,16 +23328,16 @@
         <v>28</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F62" s="8"/>
     </row>
@@ -22445,16 +23346,16 @@
         <v>28</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F63" s="8"/>
     </row>
@@ -22463,18 +23364,54 @@
         <v>28</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F64" s="8"/>
+    </row>
+    <row r="65" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="E65" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="F65" s="8"/>
+    </row>
+    <row r="66" customFormat="false" ht="86.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C66" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="E66" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="F66" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -22495,7 +23432,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -22506,24 +23443,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>50</v>
@@ -22536,7 +23473,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22554,7 +23491,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22572,7 +23509,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22590,7 +23527,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22608,7 +23545,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22626,7 +23563,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22644,7 +23581,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22662,7 +23599,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22680,7 +23617,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22698,7 +23635,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22716,7 +23653,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22734,7 +23671,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22752,7 +23689,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22770,7 +23707,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22788,7 +23725,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22806,7 +23743,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22824,7 +23761,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22842,7 +23779,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22860,7 +23797,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22878,7 +23815,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22896,7 +23833,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22914,7 +23851,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22932,7 +23869,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22950,7 +23887,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22968,7 +23905,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22986,7 +23923,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23004,7 +23941,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23022,7 +23959,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23040,7 +23977,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23058,7 +23995,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23076,7 +24013,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23094,7 +24031,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23112,7 +24049,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23130,7 +24067,7 @@
         <v>1</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23148,7 +24085,25 @@
         <v>1</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>336</v>
+        <v>344</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" s="8" t="n">
+        <v>112</v>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>112</v>
+      </c>
+      <c r="D37" s="10" t="n">
+        <f aca="false">IFERROR(C37/B37,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>